<commit_message>
Update arbeidsplan Excel from SharePoint
</commit_message>
<xml_diff>
--- a/input/Arbeidsplan simulatoroperatører.xlsx
+++ b/input/Arbeidsplan simulatoroperatører.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://avinor.sharepoint.com/sites/GRP_Simulatordrift_avd.Vaernes/Delte dokumenter/General/Arbeidsplaner/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6568" documentId="8_{95B923E9-95EE-4F78-B225-2EDB4F75667E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{475D40F1-0C6E-4158-ABD3-C073EBD2B35E}"/>
+  <xr:revisionPtr revIDLastSave="6593" documentId="8_{95B923E9-95EE-4F78-B225-2EDB4F75667E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9DC5B5A8-1242-4926-A273-DCE4B3B1E325}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="lgNItpb0Ti65q+mfEUdHXTOz24BuywDWtkFml2UWap2uCRRSwJcP050KCJ16GV7eXwgKeIkDdd7RYQr9U+X8Rw==" workbookSaltValue="526Uxco+d+5gCLKuUY2fsw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Uke 1-6" sheetId="7" r:id="rId1"/>
@@ -75,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4785" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4792" uniqueCount="359">
   <si>
     <t>Uke 01</t>
   </si>
@@ -947,9 +947,6 @@
     <t>SF EV 4</t>
   </si>
   <si>
-    <t>SE ZV 4</t>
-  </si>
-  <si>
     <t>Uke 38</t>
   </si>
   <si>
@@ -1031,9 +1028,6 @@
     <t>9 SE AFIS gr. Utd</t>
   </si>
   <si>
-    <t>SE EV 1</t>
-  </si>
-  <si>
     <t>Uke 43</t>
   </si>
   <si>
@@ -1146,6 +1140,18 @@
   </si>
   <si>
     <t>9 SF KUT SUR OV</t>
+  </si>
+  <si>
+    <t>SE ZV 4 BH</t>
+  </si>
+  <si>
+    <t>SE ZV 4 MVO</t>
+  </si>
+  <si>
+    <t>SE EV 1 OFF</t>
+  </si>
+  <si>
+    <t>SF BR 4 GG</t>
   </si>
 </sst>
 </file>
@@ -20971,10 +20977,10 @@
       <c r="N4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="O4" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="P4" s="21"/>
+      <c r="O4" s="36" t="s">
+        <v>277</v>
+      </c>
+      <c r="P4" s="37"/>
       <c r="Q4" s="50" t="s">
         <v>275</v>
       </c>
@@ -21451,14 +21457,14 @@
       <c r="N14" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="O14" s="36" t="s">
-        <v>277</v>
-      </c>
-      <c r="P14" s="37"/>
-      <c r="Q14" s="36" t="s">
-        <v>277</v>
-      </c>
-      <c r="R14" s="37"/>
+      <c r="O14" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="P14" s="41"/>
+      <c r="Q14" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="R14" s="41"/>
       <c r="S14" s="36" t="s">
         <v>277</v>
       </c>
@@ -21580,8 +21586,12 @@
       <c r="I17" s="5"/>
       <c r="J17" s="5"/>
       <c r="K17" s="5"/>
+      <c r="Q17" s="36" t="s">
+        <v>358</v>
+      </c>
+      <c r="R17" s="37"/>
       <c r="S17" s="46" t="s">
-        <v>290</v>
+        <v>355</v>
       </c>
       <c r="T17" s="47"/>
     </row>
@@ -21598,7 +21608,7 @@
       <c r="J18" s="5"/>
       <c r="K18" s="5"/>
       <c r="S18" s="46" t="s">
-        <v>290</v>
+        <v>356</v>
       </c>
       <c r="T18" s="47"/>
     </row>
@@ -21630,7 +21640,7 @@
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>1</v>
@@ -21663,7 +21673,7 @@
         <v>46283</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="O21" s="2" t="s">
         <v>1</v>
@@ -21757,11 +21767,11 @@
       </c>
       <c r="E23" s="21"/>
       <c r="F23" s="24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="G23" s="25"/>
       <c r="H23" s="24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="I23" s="25"/>
       <c r="J23" s="36" t="s">
@@ -21805,11 +21815,11 @@
       </c>
       <c r="E24" s="29"/>
       <c r="F24" s="24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G24" s="25"/>
       <c r="H24" s="24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="I24" s="25"/>
       <c r="J24" s="40" t="s">
@@ -21868,7 +21878,7 @@
         <v>21</v>
       </c>
       <c r="O25" s="26" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="P25" s="27"/>
       <c r="Q25" s="34" t="s">
@@ -21993,38 +22003,38 @@
       </c>
       <c r="C28" s="21"/>
       <c r="D28" s="24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E28" s="25"/>
       <c r="F28" s="26" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G28" s="27"/>
       <c r="H28" s="26" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="I28" s="27"/>
       <c r="J28" s="26" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="K28" s="27"/>
       <c r="N28" s="6" t="s">
         <v>28</v>
       </c>
       <c r="O28" s="26" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="P28" s="27"/>
       <c r="Q28" s="26" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="R28" s="27"/>
       <c r="S28" s="26" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="T28" s="27"/>
       <c r="U28" s="26" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="V28" s="27"/>
       <c r="W28" s="20" t="s">
@@ -22097,7 +22107,7 @@
       </c>
       <c r="G30" s="45"/>
       <c r="H30" s="52" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="I30" s="53"/>
       <c r="J30" s="44" t="s">
@@ -22112,7 +22122,7 @@
       </c>
       <c r="P30" s="45"/>
       <c r="Q30" s="32" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="R30" s="33"/>
       <c r="S30" s="44" t="s">
@@ -22133,23 +22143,23 @@
         <v>37</v>
       </c>
       <c r="B31" s="24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C31" s="25"/>
       <c r="D31" s="24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E31" s="25"/>
       <c r="F31" s="26" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G31" s="27"/>
       <c r="H31" s="26" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="I31" s="27"/>
       <c r="J31" s="26" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K31" s="27"/>
       <c r="L31" s="7"/>
@@ -22158,23 +22168,23 @@
         <v>37</v>
       </c>
       <c r="O31" s="26" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="P31" s="27"/>
       <c r="Q31" s="26" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="R31" s="27"/>
       <c r="S31" s="26" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="T31" s="27"/>
       <c r="U31" s="26" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="V31" s="27"/>
       <c r="W31" s="32" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="X31" s="33"/>
     </row>
@@ -22249,7 +22259,7 @@
       </c>
       <c r="I33" s="31"/>
       <c r="J33" s="24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="K33" s="25"/>
       <c r="L33" s="7"/>
@@ -22258,23 +22268,23 @@
         <v>45</v>
       </c>
       <c r="O33" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="P33" s="35"/>
       <c r="Q33" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="R33" s="35"/>
       <c r="S33" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="T33" s="35"/>
       <c r="U33" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="V33" s="35"/>
       <c r="W33" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="X33" s="35"/>
     </row>
@@ -22283,7 +22293,7 @@
         <v>48</v>
       </c>
       <c r="B34" s="24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C34" s="25"/>
       <c r="D34" s="36" t="s">
@@ -22349,7 +22359,7 @@
       </c>
       <c r="I35" s="47"/>
       <c r="J35" s="24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="K35" s="25"/>
       <c r="L35" s="7"/>
@@ -22362,15 +22372,15 @@
       </c>
       <c r="P35" s="37"/>
       <c r="Q35" s="34" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="R35" s="35"/>
       <c r="S35" s="34" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="T35" s="35"/>
       <c r="U35" s="34" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="V35" s="35"/>
       <c r="W35" s="34" t="s">
@@ -22412,7 +22422,7 @@
       </c>
       <c r="P36" s="21"/>
       <c r="Q36" s="32" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="R36" s="33"/>
       <c r="S36" s="34" t="s">
@@ -22424,7 +22434,7 @@
       </c>
       <c r="V36" s="37"/>
       <c r="W36" s="32" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="X36" s="33"/>
     </row>
@@ -22518,7 +22528,7 @@
     </row>
     <row r="40" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>1</v>
@@ -22553,7 +22563,7 @@
       <c r="L40" s="7"/>
       <c r="M40" s="7"/>
       <c r="N40" s="1" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="O40" s="2" t="s">
         <v>1</v>
@@ -22641,11 +22651,11 @@
         <v>10</v>
       </c>
       <c r="B42" s="24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C42" s="25"/>
       <c r="D42" s="24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E42" s="25"/>
       <c r="F42" s="20" t="s">
@@ -22670,7 +22680,7 @@
       </c>
       <c r="P42" s="37"/>
       <c r="Q42" s="36" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="R42" s="37"/>
       <c r="S42" s="36" t="s">
@@ -22691,11 +22701,11 @@
         <v>15</v>
       </c>
       <c r="B43" s="26" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C43" s="27"/>
       <c r="D43" s="26" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E43" s="27"/>
       <c r="F43" s="20" t="s">
@@ -22703,11 +22713,11 @@
       </c>
       <c r="G43" s="21"/>
       <c r="H43" s="26" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="I43" s="27"/>
       <c r="J43" s="24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="K43" s="25"/>
       <c r="L43" s="7"/>
@@ -22720,7 +22730,7 @@
       </c>
       <c r="P43" s="37"/>
       <c r="Q43" s="36" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="R43" s="37"/>
       <c r="S43" s="36" t="s">
@@ -22728,7 +22738,7 @@
       </c>
       <c r="T43" s="37"/>
       <c r="U43" s="54" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="V43" s="55"/>
       <c r="W43" s="20" t="s">
@@ -22766,19 +22776,19 @@
         <v>21</v>
       </c>
       <c r="O44" s="26" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="P44" s="27"/>
       <c r="Q44" s="26" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="R44" s="27"/>
       <c r="S44" s="22" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="T44" s="23"/>
       <c r="U44" s="54" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="V44" s="55"/>
       <c r="W44" s="36" t="s">
@@ -22855,14 +22865,14 @@
       </c>
       <c r="I46" s="47"/>
       <c r="J46" s="34" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="K46" s="35"/>
       <c r="N46" s="6" t="s">
         <v>26</v>
       </c>
       <c r="O46" s="34" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="P46" s="35"/>
       <c r="Q46" s="34" t="s">
@@ -22887,11 +22897,11 @@
         <v>28</v>
       </c>
       <c r="B47" s="26" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C47" s="27"/>
       <c r="D47" s="26" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E47" s="27"/>
       <c r="F47" s="36" t="s">
@@ -22899,22 +22909,22 @@
       </c>
       <c r="G47" s="37"/>
       <c r="H47" s="26" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="I47" s="27"/>
       <c r="J47" s="24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="K47" s="25"/>
       <c r="N47" s="6" t="s">
         <v>28</v>
       </c>
       <c r="O47" s="26" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="P47" s="27"/>
       <c r="Q47" s="26" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="R47" s="27"/>
       <c r="S47" s="34" t="s">
@@ -22962,19 +22972,19 @@
       </c>
       <c r="P48" s="21"/>
       <c r="Q48" s="54" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="R48" s="55"/>
       <c r="S48" s="54" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="T48" s="55"/>
       <c r="U48" s="46" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="V48" s="47"/>
       <c r="W48" s="54" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="X48" s="55"/>
     </row>
@@ -22983,15 +22993,15 @@
         <v>35</v>
       </c>
       <c r="B49" s="24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C49" s="25"/>
       <c r="D49" s="24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E49" s="25"/>
       <c r="F49" s="44" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="G49" s="45"/>
       <c r="H49" s="46" t="s">
@@ -22999,7 +23009,7 @@
       </c>
       <c r="I49" s="47"/>
       <c r="J49" s="44" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="K49" s="45"/>
       <c r="N49" s="6" t="s">
@@ -23058,19 +23068,19 @@
       </c>
       <c r="P50" s="35"/>
       <c r="Q50" s="54" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="R50" s="55"/>
       <c r="S50" s="54" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="T50" s="55"/>
       <c r="U50" s="46" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="V50" s="47"/>
       <c r="W50" s="54" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="X50" s="55"/>
     </row>
@@ -23106,15 +23116,15 @@
       </c>
       <c r="P51" s="45"/>
       <c r="Q51" s="34" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="R51" s="35"/>
       <c r="S51" s="34" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="T51" s="35"/>
       <c r="U51" s="46" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="V51" s="47"/>
       <c r="W51" s="44" t="s">
@@ -23135,38 +23145,38 @@
       </c>
       <c r="E52" s="23"/>
       <c r="F52" s="24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G52" s="25"/>
       <c r="H52" s="24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="I52" s="25"/>
       <c r="J52" s="34" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="K52" s="35"/>
       <c r="N52" s="12" t="s">
         <v>45</v>
       </c>
       <c r="O52" s="34" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="P52" s="35"/>
       <c r="Q52" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="R52" s="35"/>
       <c r="S52" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="T52" s="35"/>
       <c r="U52" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="V52" s="35"/>
       <c r="W52" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="X52" s="35"/>
     </row>
@@ -23198,7 +23208,7 @@
         <v>48</v>
       </c>
       <c r="O53" s="34" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="P53" s="35"/>
       <c r="Q53" s="34" t="s">
@@ -23231,11 +23241,11 @@
       </c>
       <c r="E54" s="47"/>
       <c r="F54" s="24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="G54" s="25"/>
       <c r="H54" s="24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="I54" s="25"/>
       <c r="J54" s="46" t="s">
@@ -23339,7 +23349,7 @@
       </c>
       <c r="K56" s="23"/>
       <c r="S56" s="22" t="s">
-        <v>318</v>
+        <v>357</v>
       </c>
       <c r="T56" s="23"/>
     </row>
@@ -23464,8 +23474,9 @@
       <c r="X66" s="5"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="D/sbAv5uAPXBcgTGv2GcdOcmJHp1lnRyUbjcBHiVNmcnSXDKs8qTCxAiCrVywBeN3gEU8QTnMoCm7UvMzGWrUQ==" saltValue="izdUJKiIdN/ZR9tRIXeQhg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
-  <mergeCells count="468">
+  <mergeCells count="469">
+    <mergeCell ref="Q17:R17"/>
+    <mergeCell ref="O8:P8"/>
     <mergeCell ref="S18:T18"/>
     <mergeCell ref="S56:T56"/>
     <mergeCell ref="W54:X54"/>
@@ -23811,7 +23822,6 @@
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="H3:I3"/>
     <mergeCell ref="J3:K3"/>
-    <mergeCell ref="O4:P4"/>
     <mergeCell ref="O7:P7"/>
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="S3:T3"/>
@@ -23840,7 +23850,7 @@
     <mergeCell ref="S6:T6"/>
     <mergeCell ref="O10:P10"/>
     <mergeCell ref="O9:P9"/>
-    <mergeCell ref="O8:P8"/>
+    <mergeCell ref="O4:P4"/>
     <mergeCell ref="S13:T13"/>
     <mergeCell ref="U13:V13"/>
     <mergeCell ref="U30:V30"/>
@@ -23952,7 +23962,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:X60"/>
+  <dimension ref="A1:X61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9" style="4" bestFit="1" customWidth="1"/>
@@ -23985,7 +23995,7 @@
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -24018,7 +24028,7 @@
         <v>46318</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="O1" s="2" t="s">
         <v>1</v>
@@ -24072,7 +24082,7 @@
       </c>
       <c r="I2" s="39"/>
       <c r="J2" s="34" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="K2" s="35"/>
       <c r="N2" s="1" t="s">
@@ -24087,11 +24097,11 @@
       </c>
       <c r="R2" s="39"/>
       <c r="S2" s="38" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="T2" s="39"/>
       <c r="U2" s="38" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="V2" s="39"/>
       <c r="W2" s="38" t="s">
@@ -24135,7 +24145,7 @@
       </c>
       <c r="R3" s="21"/>
       <c r="S3" s="105" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="T3" s="106"/>
       <c r="U3" s="20" t="s">
@@ -24152,11 +24162,11 @@
         <v>15</v>
       </c>
       <c r="B4" s="76" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="C4" s="77"/>
       <c r="D4" s="76" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="E4" s="77"/>
       <c r="F4" s="20" t="s">
@@ -24164,11 +24174,11 @@
       </c>
       <c r="G4" s="21"/>
       <c r="H4" s="76" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="I4" s="77"/>
       <c r="J4" s="76" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="K4" s="77"/>
       <c r="N4" s="1" t="s">
@@ -24191,7 +24201,7 @@
       </c>
       <c r="V4" s="43"/>
       <c r="W4" s="24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="X4" s="25"/>
     </row>
@@ -24200,11 +24210,11 @@
         <v>21</v>
       </c>
       <c r="B5" s="76" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C5" s="77"/>
       <c r="D5" s="76" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="E5" s="77"/>
       <c r="F5" s="36" t="s">
@@ -24223,23 +24233,23 @@
         <v>21</v>
       </c>
       <c r="O5" s="34" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="P5" s="35"/>
       <c r="Q5" s="34" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="R5" s="35"/>
       <c r="S5" s="34" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="T5" s="35"/>
       <c r="U5" s="34" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="V5" s="35"/>
       <c r="W5" s="34" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="X5" s="35"/>
     </row>
@@ -24323,11 +24333,11 @@
       </c>
       <c r="P7" s="33"/>
       <c r="Q7" s="24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="R7" s="25"/>
       <c r="S7" s="105" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="T7" s="106"/>
       <c r="U7" s="20" t="s">
@@ -24356,11 +24366,11 @@
       </c>
       <c r="G8" s="21"/>
       <c r="H8" s="34" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="I8" s="35"/>
       <c r="J8" s="34" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="K8" s="35"/>
       <c r="L8" s="7"/>
@@ -24369,23 +24379,23 @@
         <v>28</v>
       </c>
       <c r="O8" s="34" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="P8" s="35"/>
       <c r="Q8" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="R8" s="35"/>
       <c r="S8" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="T8" s="35"/>
       <c r="U8" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="V8" s="35"/>
       <c r="W8" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="X8" s="35"/>
     </row>
@@ -24394,23 +24404,23 @@
         <v>32</v>
       </c>
       <c r="B9" s="34" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C9" s="35"/>
       <c r="D9" s="34" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="E9" s="35"/>
       <c r="F9" s="34" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="G9" s="35"/>
       <c r="H9" s="34" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="I9" s="35"/>
       <c r="J9" s="34" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="K9" s="35"/>
       <c r="L9" s="7"/>
@@ -24419,23 +24429,23 @@
         <v>32</v>
       </c>
       <c r="O9" s="24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="P9" s="25"/>
       <c r="Q9" s="24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="R9" s="25"/>
       <c r="S9" s="24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="T9" s="25"/>
       <c r="U9" s="24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="V9" s="25"/>
       <c r="W9" s="24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="X9" s="25"/>
     </row>
@@ -24452,7 +24462,7 @@
       </c>
       <c r="E10" s="21"/>
       <c r="F10" s="34" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="G10" s="35"/>
       <c r="H10" s="20" t="s">
@@ -24469,7 +24479,7 @@
         <v>35</v>
       </c>
       <c r="O10" s="24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="P10" s="25"/>
       <c r="Q10" s="20" t="s">
@@ -24477,7 +24487,7 @@
       </c>
       <c r="R10" s="21"/>
       <c r="S10" s="24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="T10" s="25"/>
       <c r="U10" s="20" t="s">
@@ -24529,7 +24539,7 @@
       </c>
       <c r="T11" s="47"/>
       <c r="U11" s="24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="V11" s="25"/>
       <c r="W11" s="20" t="s">
@@ -24546,7 +24556,7 @@
       </c>
       <c r="C12" s="21"/>
       <c r="D12" s="34" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="E12" s="35"/>
       <c r="F12" s="34" t="s">
@@ -24565,7 +24575,7 @@
         <v>40</v>
       </c>
       <c r="O12" s="34" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="P12" s="35"/>
       <c r="Q12" s="34" t="s">
@@ -24594,19 +24604,19 @@
       </c>
       <c r="C13" s="35"/>
       <c r="D13" s="44" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="E13" s="45"/>
       <c r="F13" s="34" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="G13" s="35"/>
       <c r="H13" s="34" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="I13" s="35"/>
       <c r="J13" s="34" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="K13" s="35"/>
       <c r="N13" s="12" t="s">
@@ -24654,14 +24664,14 @@
       </c>
       <c r="I14" s="37"/>
       <c r="J14" s="34" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="K14" s="35"/>
       <c r="N14" s="1" t="s">
         <v>48</v>
       </c>
       <c r="O14" s="34" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="P14" s="35"/>
       <c r="Q14" s="34" t="s">
@@ -24686,11 +24696,11 @@
         <v>49</v>
       </c>
       <c r="B15" s="34" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="C15" s="35"/>
       <c r="D15" s="34" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="E15" s="35"/>
       <c r="F15" s="36" t="s">
@@ -24721,7 +24731,7 @@
       </c>
       <c r="T15" s="47"/>
       <c r="U15" s="105" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="V15" s="106"/>
       <c r="W15" s="20" t="s">
@@ -24746,11 +24756,11 @@
       </c>
       <c r="G16" s="47"/>
       <c r="H16" s="76" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="I16" s="77"/>
       <c r="J16" s="76" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="K16" s="77"/>
       <c r="N16" s="1" t="s">
@@ -24769,7 +24779,7 @@
       </c>
       <c r="T16" s="47"/>
       <c r="U16" s="105" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="V16" s="106"/>
       <c r="W16" s="20" t="s">
@@ -24824,7 +24834,7 @@
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>1</v>
@@ -24857,7 +24867,7 @@
         <v>46325</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="O19" s="2" t="s">
         <v>1</v>
@@ -24951,11 +24961,11 @@
       </c>
       <c r="E21" s="21"/>
       <c r="F21" s="78" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="G21" s="79"/>
       <c r="H21" s="78" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="I21" s="79"/>
       <c r="J21" s="20" t="s">
@@ -24966,15 +24976,15 @@
         <v>10</v>
       </c>
       <c r="O21" s="24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="P21" s="25"/>
       <c r="Q21" s="24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="R21" s="25"/>
       <c r="S21" s="24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="T21" s="25"/>
       <c r="U21" s="20" t="s">
@@ -25014,23 +25024,23 @@
         <v>15</v>
       </c>
       <c r="O22" s="24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="P22" s="25"/>
       <c r="Q22" s="24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="R22" s="25"/>
       <c r="S22" s="24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="T22" s="25"/>
       <c r="U22" s="24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="V22" s="25"/>
       <c r="W22" s="24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="X22" s="25"/>
     </row>
@@ -25039,7 +25049,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="34" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C23" s="35"/>
       <c r="D23" s="34" t="s">
@@ -25062,7 +25072,7 @@
         <v>21</v>
       </c>
       <c r="O23" s="46" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="P23" s="47"/>
       <c r="Q23" s="34" t="s">
@@ -25074,11 +25084,11 @@
       </c>
       <c r="T23" s="35"/>
       <c r="U23" s="24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="V23" s="25"/>
       <c r="W23" s="24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="X23" s="25"/>
     </row>
@@ -25162,15 +25172,15 @@
       </c>
       <c r="P25" s="47"/>
       <c r="Q25" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="R25" s="35"/>
       <c r="S25" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="T25" s="35"/>
       <c r="U25" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="V25" s="35"/>
       <c r="W25" s="46" t="s">
@@ -25187,11 +25197,11 @@
       </c>
       <c r="C26" s="21"/>
       <c r="D26" s="44" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="E26" s="45"/>
       <c r="F26" s="44" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="G26" s="45"/>
       <c r="H26" s="20" t="s">
@@ -25199,7 +25209,7 @@
       </c>
       <c r="I26" s="21"/>
       <c r="J26" s="78" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="K26" s="79"/>
       <c r="L26" s="7"/>
@@ -25208,15 +25218,15 @@
         <v>28</v>
       </c>
       <c r="O26" s="105" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="P26" s="106"/>
       <c r="Q26" s="105" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="R26" s="106"/>
       <c r="S26" s="105" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="T26" s="106"/>
       <c r="U26" s="46" t="s">
@@ -25224,7 +25234,7 @@
       </c>
       <c r="V26" s="47"/>
       <c r="W26" s="105" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="X26" s="106"/>
     </row>
@@ -25249,7 +25259,7 @@
       </c>
       <c r="I27" s="21"/>
       <c r="J27" s="78" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="K27" s="79"/>
       <c r="L27" s="7"/>
@@ -25257,24 +25267,24 @@
       <c r="N27" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="O27" s="34" t="s">
-        <v>350</v>
-      </c>
-      <c r="P27" s="35"/>
+      <c r="O27" s="46" t="s">
+        <v>31</v>
+      </c>
+      <c r="P27" s="47"/>
       <c r="Q27" s="34" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="R27" s="35"/>
       <c r="S27" s="34" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="T27" s="35"/>
       <c r="U27" s="34" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="V27" s="35"/>
       <c r="W27" s="34" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="X27" s="35"/>
     </row>
@@ -25291,11 +25301,11 @@
       </c>
       <c r="E28" s="23"/>
       <c r="F28" s="78" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="G28" s="79"/>
       <c r="H28" s="78" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="I28" s="79"/>
       <c r="J28" s="20" t="s">
@@ -25333,23 +25343,23 @@
         <v>37</v>
       </c>
       <c r="B29" s="34" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C29" s="35"/>
       <c r="D29" s="34" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="E29" s="35"/>
       <c r="F29" s="34" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="G29" s="35"/>
       <c r="H29" s="34" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="I29" s="35"/>
       <c r="J29" s="34" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="K29" s="35"/>
       <c r="L29" s="7"/>
@@ -25358,23 +25368,23 @@
         <v>37</v>
       </c>
       <c r="O29" s="34" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="P29" s="35"/>
       <c r="Q29" s="34" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="R29" s="35"/>
       <c r="S29" s="34" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="T29" s="35"/>
       <c r="U29" s="34" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="V29" s="35"/>
       <c r="W29" s="34" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="X29" s="35"/>
     </row>
@@ -25433,23 +25443,23 @@
         <v>45</v>
       </c>
       <c r="B31" s="34" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C31" s="35"/>
       <c r="D31" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="E31" s="35"/>
       <c r="F31" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G31" s="35"/>
       <c r="H31" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="I31" s="35"/>
       <c r="J31" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="K31" s="35"/>
       <c r="L31" s="7"/>
@@ -25483,7 +25493,7 @@
         <v>48</v>
       </c>
       <c r="B32" s="34" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C32" s="35"/>
       <c r="D32" s="22" t="s">
@@ -25507,10 +25517,10 @@
       <c r="N32" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="O32" s="46" t="s">
-        <v>44</v>
-      </c>
-      <c r="P32" s="47"/>
+      <c r="O32" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="P32" s="41"/>
       <c r="Q32" s="34" t="s">
         <v>103</v>
       </c>
@@ -25533,11 +25543,11 @@
         <v>49</v>
       </c>
       <c r="B33" s="34" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="C33" s="35"/>
       <c r="D33" s="34" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="E33" s="35"/>
       <c r="F33" s="34" t="s">
@@ -25608,15 +25618,15 @@
         <v>50</v>
       </c>
       <c r="O34" s="105" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="P34" s="106"/>
       <c r="Q34" s="105" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="R34" s="106"/>
       <c r="S34" s="105" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="T34" s="106"/>
       <c r="U34" s="20" t="s">
@@ -25624,7 +25634,7 @@
       </c>
       <c r="V34" s="21"/>
       <c r="W34" s="105" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="X34" s="106"/>
     </row>
@@ -25642,168 +25652,141 @@
       <c r="K35" s="9"/>
       <c r="L35" s="7"/>
       <c r="M35" s="7"/>
-      <c r="O35" s="9"/>
-      <c r="P35" s="9"/>
+      <c r="O35" s="34" t="s">
+        <v>348</v>
+      </c>
+      <c r="P35" s="35"/>
       <c r="U35" s="9"/>
       <c r="V35" s="9"/>
       <c r="W35" s="9"/>
       <c r="X35" s="9"/>
     </row>
-    <row r="36" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A36" s="7"/>
-      <c r="B36" s="7"/>
-      <c r="C36" s="7"/>
-      <c r="D36" s="7"/>
-      <c r="E36" s="7"/>
-      <c r="F36" s="7"/>
-      <c r="G36" s="7"/>
-      <c r="H36" s="7"/>
-      <c r="I36" s="7"/>
-      <c r="J36" s="7"/>
-      <c r="K36" s="7"/>
+    <row r="36" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="5"/>
+      <c r="B36" s="9"/>
+      <c r="C36" s="9"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
+      <c r="I36" s="9"/>
+      <c r="J36" s="9"/>
+      <c r="K36" s="9"/>
       <c r="L36" s="7"/>
       <c r="M36" s="7"/>
+      <c r="O36" s="9"/>
+      <c r="P36" s="9"/>
+      <c r="U36" s="9"/>
+      <c r="V36" s="9"/>
+      <c r="W36" s="9"/>
+      <c r="X36" s="9"/>
     </row>
     <row r="37" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A37" s="1" t="s">
-        <v>333</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C37" s="3">
-        <v>46328</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E37" s="3">
-        <v>46329</v>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="G37" s="3">
-        <v>46330</v>
-      </c>
-      <c r="H37" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="I37" s="3">
-        <v>46331</v>
-      </c>
-      <c r="J37" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="K37" s="3">
-        <v>46332</v>
-      </c>
+      <c r="A37" s="7"/>
+      <c r="B37" s="7"/>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="7"/>
+      <c r="G37" s="7"/>
+      <c r="H37" s="7"/>
+      <c r="I37" s="7"/>
+      <c r="J37" s="7"/>
+      <c r="K37" s="7"/>
       <c r="L37" s="7"/>
       <c r="M37" s="7"/>
-      <c r="N37" s="1" t="s">
-        <v>334</v>
-      </c>
-      <c r="O37" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="P37" s="3">
-        <v>46349</v>
-      </c>
-      <c r="Q37" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="R37" s="3">
-        <v>46350</v>
-      </c>
-      <c r="S37" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="T37" s="3">
-        <v>46351</v>
-      </c>
-      <c r="U37" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="V37" s="3">
-        <v>46352</v>
-      </c>
-      <c r="W37" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="X37" s="3">
-        <v>46353</v>
-      </c>
     </row>
     <row r="38" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B38" s="38" t="s">
-        <v>9</v>
-      </c>
-      <c r="C38" s="39"/>
-      <c r="D38" s="38" t="s">
-        <v>9</v>
-      </c>
-      <c r="E38" s="39"/>
-      <c r="F38" s="38" t="s">
-        <v>335</v>
-      </c>
-      <c r="G38" s="39"/>
-      <c r="H38" s="38" t="s">
-        <v>9</v>
-      </c>
-      <c r="I38" s="39"/>
-      <c r="J38" s="34" t="s">
-        <v>92</v>
-      </c>
-      <c r="K38" s="35"/>
+        <v>331</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C38" s="3">
+        <v>46328</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E38" s="3">
+        <v>46329</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G38" s="3">
+        <v>46330</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I38" s="3">
+        <v>46331</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="K38" s="3">
+        <v>46332</v>
+      </c>
       <c r="L38" s="7"/>
       <c r="M38" s="7"/>
       <c r="N38" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="O38" s="38" t="s">
-        <v>9</v>
-      </c>
-      <c r="P38" s="39"/>
-      <c r="Q38" s="38" t="s">
-        <v>9</v>
-      </c>
-      <c r="R38" s="39"/>
-      <c r="S38" s="38" t="s">
-        <v>9</v>
-      </c>
-      <c r="T38" s="39"/>
-      <c r="U38" s="38" t="s">
-        <v>9</v>
-      </c>
-      <c r="V38" s="39"/>
-      <c r="W38" s="38" t="s">
-        <v>9</v>
-      </c>
-      <c r="X38" s="39"/>
+        <v>332</v>
+      </c>
+      <c r="O38" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="P38" s="3">
+        <v>46349</v>
+      </c>
+      <c r="Q38" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="R38" s="3">
+        <v>46350</v>
+      </c>
+      <c r="S38" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="T38" s="3">
+        <v>46351</v>
+      </c>
+      <c r="U38" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="V38" s="3">
+        <v>46352</v>
+      </c>
+      <c r="W38" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="X38" s="3">
+        <v>46353</v>
+      </c>
     </row>
     <row r="39" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B39" s="34" t="s">
-        <v>336</v>
-      </c>
-      <c r="C39" s="35"/>
-      <c r="D39" s="34" t="s">
-        <v>336</v>
-      </c>
-      <c r="E39" s="35"/>
-      <c r="F39" s="34" t="s">
-        <v>336</v>
-      </c>
-      <c r="G39" s="35"/>
-      <c r="H39" s="34" t="s">
-        <v>336</v>
-      </c>
-      <c r="I39" s="35"/>
+        <v>7</v>
+      </c>
+      <c r="B39" s="38" t="s">
+        <v>9</v>
+      </c>
+      <c r="C39" s="39"/>
+      <c r="D39" s="38" t="s">
+        <v>9</v>
+      </c>
+      <c r="E39" s="39"/>
+      <c r="F39" s="38" t="s">
+        <v>333</v>
+      </c>
+      <c r="G39" s="39"/>
+      <c r="H39" s="38" t="s">
+        <v>9</v>
+      </c>
+      <c r="I39" s="39"/>
       <c r="J39" s="34" t="s">
         <v>92</v>
       </c>
@@ -25811,118 +25794,120 @@
       <c r="L39" s="7"/>
       <c r="M39" s="7"/>
       <c r="N39" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="O39" s="38" t="s">
+        <v>9</v>
+      </c>
+      <c r="P39" s="39"/>
+      <c r="Q39" s="38" t="s">
+        <v>9</v>
+      </c>
+      <c r="R39" s="39"/>
+      <c r="S39" s="38" t="s">
+        <v>9</v>
+      </c>
+      <c r="T39" s="39"/>
+      <c r="U39" s="38" t="s">
+        <v>9</v>
+      </c>
+      <c r="V39" s="39"/>
+      <c r="W39" s="38" t="s">
+        <v>9</v>
+      </c>
+      <c r="X39" s="39"/>
+    </row>
+    <row r="40" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A40" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="O39" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="P39" s="21"/>
-      <c r="Q39" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="R39" s="21"/>
-      <c r="S39" s="98" t="s">
+      <c r="B40" s="34" t="s">
+        <v>334</v>
+      </c>
+      <c r="C40" s="35"/>
+      <c r="D40" s="34" t="s">
+        <v>334</v>
+      </c>
+      <c r="E40" s="35"/>
+      <c r="F40" s="34" t="s">
+        <v>334</v>
+      </c>
+      <c r="G40" s="35"/>
+      <c r="H40" s="34" t="s">
+        <v>334</v>
+      </c>
+      <c r="I40" s="35"/>
+      <c r="J40" s="34" t="s">
+        <v>92</v>
+      </c>
+      <c r="K40" s="35"/>
+      <c r="L40" s="7"/>
+      <c r="M40" s="7"/>
+      <c r="N40" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="O40" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="P40" s="21"/>
+      <c r="Q40" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="R40" s="21"/>
+      <c r="S40" s="98" t="s">
         <v>219</v>
       </c>
-      <c r="T39" s="99"/>
-      <c r="U39" s="98" t="s">
+      <c r="T40" s="99"/>
+      <c r="U40" s="98" t="s">
         <v>220</v>
       </c>
-      <c r="V39" s="99"/>
-      <c r="W39" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="X39" s="21"/>
-    </row>
-    <row r="40" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="1" t="s">
+      <c r="V40" s="99"/>
+      <c r="W40" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="X40" s="21"/>
+    </row>
+    <row r="41" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B40" s="34" t="s">
-        <v>312</v>
-      </c>
-      <c r="C40" s="35"/>
-      <c r="D40" s="42" t="s">
+      <c r="B41" s="34" t="s">
+        <v>311</v>
+      </c>
+      <c r="C41" s="35"/>
+      <c r="D41" s="42" t="s">
         <v>72</v>
       </c>
-      <c r="E40" s="43"/>
-      <c r="F40" s="46" t="s">
+      <c r="E41" s="43"/>
+      <c r="F41" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="G40" s="47"/>
-      <c r="H40" s="46" t="s">
+      <c r="G41" s="47"/>
+      <c r="H41" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="I40" s="47"/>
-      <c r="J40" s="46" t="s">
+      <c r="I41" s="47"/>
+      <c r="J41" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="K40" s="47"/>
-      <c r="N40" s="1" t="s">
+      <c r="K41" s="47"/>
+      <c r="N41" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="O40" s="46" t="s">
+      <c r="O41" s="46" t="s">
         <v>31</v>
-      </c>
-      <c r="P40" s="47"/>
-      <c r="Q40" s="46" t="s">
-        <v>31</v>
-      </c>
-      <c r="R40" s="47"/>
-      <c r="S40" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="T40" s="21"/>
-      <c r="U40" s="98" t="s">
-        <v>219</v>
-      </c>
-      <c r="V40" s="99"/>
-      <c r="W40" s="46" t="s">
-        <v>31</v>
-      </c>
-      <c r="X40" s="47"/>
-    </row>
-    <row r="41" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A41" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B41" s="46" t="s">
-        <v>44</v>
-      </c>
-      <c r="C41" s="47"/>
-      <c r="D41" s="34" t="s">
-        <v>103</v>
-      </c>
-      <c r="E41" s="35"/>
-      <c r="F41" s="34" t="s">
-        <v>103</v>
-      </c>
-      <c r="G41" s="35"/>
-      <c r="H41" s="34" t="s">
-        <v>103</v>
-      </c>
-      <c r="I41" s="35"/>
-      <c r="J41" s="34" t="s">
-        <v>103</v>
-      </c>
-      <c r="K41" s="35"/>
-      <c r="N41" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="O41" s="46" t="s">
-        <v>44</v>
       </c>
       <c r="P41" s="47"/>
       <c r="Q41" s="46" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="R41" s="47"/>
-      <c r="S41" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="T41" s="25"/>
+      <c r="S41" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="T41" s="21"/>
       <c r="U41" s="98" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="V41" s="99"/>
       <c r="W41" s="46" t="s">
@@ -25932,126 +25917,126 @@
     </row>
     <row r="42" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B42" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="C42" s="47"/>
+      <c r="D42" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="E42" s="35"/>
+      <c r="F42" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="G42" s="35"/>
+      <c r="H42" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="I42" s="35"/>
+      <c r="J42" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="K42" s="35"/>
+      <c r="N42" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="O42" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="P42" s="47"/>
+      <c r="Q42" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="R42" s="47"/>
+      <c r="S42" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="T42" s="25"/>
+      <c r="U42" s="98" t="s">
+        <v>215</v>
+      </c>
+      <c r="V42" s="99"/>
+      <c r="W42" s="46" t="s">
+        <v>31</v>
+      </c>
+      <c r="X42" s="47"/>
+    </row>
+    <row r="43" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A43" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B42" s="44" t="s">
+      <c r="B43" s="44" t="s">
         <v>91</v>
       </c>
-      <c r="C42" s="45"/>
-      <c r="D42" s="44" t="s">
+      <c r="C43" s="45"/>
+      <c r="D43" s="44" t="s">
         <v>91</v>
       </c>
-      <c r="E42" s="45"/>
-      <c r="F42" s="44" t="s">
+      <c r="E43" s="45"/>
+      <c r="F43" s="44" t="s">
         <v>91</v>
       </c>
-      <c r="G42" s="45"/>
-      <c r="H42" s="44" t="s">
+      <c r="G43" s="45"/>
+      <c r="H43" s="44" t="s">
         <v>91</v>
       </c>
-      <c r="I42" s="45"/>
-      <c r="J42" s="44" t="s">
+      <c r="I43" s="45"/>
+      <c r="J43" s="44" t="s">
         <v>91</v>
       </c>
-      <c r="K42" s="45"/>
-      <c r="N42" s="1" t="s">
+      <c r="K43" s="45"/>
+      <c r="N43" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="O42" s="44" t="s">
+      <c r="O43" s="44" t="s">
         <v>91</v>
       </c>
-      <c r="P42" s="45"/>
-      <c r="Q42" s="44" t="s">
+      <c r="P43" s="45"/>
+      <c r="Q43" s="44" t="s">
         <v>91</v>
       </c>
-      <c r="R42" s="45"/>
-      <c r="S42" s="44" t="s">
+      <c r="R43" s="45"/>
+      <c r="S43" s="44" t="s">
         <v>91</v>
       </c>
-      <c r="T42" s="45"/>
-      <c r="U42" s="44" t="s">
+      <c r="T43" s="45"/>
+      <c r="U43" s="44" t="s">
         <v>91</v>
       </c>
-      <c r="V42" s="45"/>
-      <c r="W42" s="44" t="s">
+      <c r="V43" s="45"/>
+      <c r="W43" s="44" t="s">
         <v>91</v>
       </c>
-      <c r="X42" s="45"/>
-    </row>
-    <row r="43" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="6" t="s">
+      <c r="X43" s="45"/>
+    </row>
+    <row r="44" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B43" s="34" t="s">
-        <v>312</v>
-      </c>
-      <c r="C43" s="35"/>
-      <c r="D43" s="50" t="s">
+      <c r="B44" s="34" t="s">
+        <v>311</v>
+      </c>
+      <c r="C44" s="35"/>
+      <c r="D44" s="50" t="s">
         <v>275</v>
       </c>
-      <c r="E43" s="51"/>
-      <c r="F43" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="G43" s="21"/>
-      <c r="H43" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="I43" s="21"/>
-      <c r="J43" s="34" t="s">
-        <v>92</v>
-      </c>
-      <c r="K43" s="35"/>
-      <c r="N43" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="O43" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="P43" s="25"/>
-      <c r="Q43" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="R43" s="25"/>
-      <c r="S43" s="24" t="s">
-        <v>19</v>
-      </c>
-      <c r="T43" s="25"/>
-      <c r="U43" s="24" t="s">
-        <v>19</v>
-      </c>
-      <c r="V43" s="25"/>
-      <c r="W43" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="X43" s="25"/>
-    </row>
-    <row r="44" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A44" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B44" s="46" t="s">
-        <v>31</v>
-      </c>
-      <c r="C44" s="47"/>
-      <c r="D44" s="34" t="s">
-        <v>337</v>
-      </c>
-      <c r="E44" s="35"/>
+      <c r="E44" s="51"/>
       <c r="F44" s="20" t="s">
         <v>9</v>
       </c>
       <c r="G44" s="21"/>
-      <c r="H44" s="46" t="s">
-        <v>31</v>
-      </c>
-      <c r="I44" s="47"/>
+      <c r="H44" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="I44" s="21"/>
       <c r="J44" s="34" t="s">
         <v>92</v>
       </c>
       <c r="K44" s="35"/>
       <c r="N44" s="6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="O44" s="24" t="s">
         <v>14</v>
@@ -26061,466 +26046,509 @@
         <v>14</v>
       </c>
       <c r="R44" s="25"/>
-      <c r="S44" s="98" t="s">
-        <v>215</v>
-      </c>
-      <c r="T44" s="99"/>
-      <c r="U44" s="98" t="s">
-        <v>217</v>
-      </c>
-      <c r="V44" s="99"/>
+      <c r="S44" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="T44" s="25"/>
+      <c r="U44" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="V44" s="25"/>
       <c r="W44" s="24" t="s">
         <v>14</v>
       </c>
       <c r="X44" s="25"/>
     </row>
-    <row r="45" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A45" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B45" s="46" t="s">
+        <v>31</v>
+      </c>
+      <c r="C45" s="47"/>
+      <c r="D45" s="34" t="s">
+        <v>335</v>
+      </c>
+      <c r="E45" s="35"/>
+      <c r="F45" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="G45" s="21"/>
+      <c r="H45" s="46" t="s">
+        <v>31</v>
+      </c>
+      <c r="I45" s="47"/>
+      <c r="J45" s="34" t="s">
+        <v>92</v>
+      </c>
+      <c r="K45" s="35"/>
+      <c r="N45" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="O45" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="P45" s="25"/>
+      <c r="Q45" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="R45" s="25"/>
+      <c r="S45" s="98" t="s">
+        <v>215</v>
+      </c>
+      <c r="T45" s="99"/>
+      <c r="U45" s="98" t="s">
+        <v>217</v>
+      </c>
+      <c r="V45" s="99"/>
+      <c r="W45" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="X45" s="25"/>
+    </row>
+    <row r="46" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B45" s="78" t="s">
-        <v>331</v>
-      </c>
-      <c r="C45" s="79"/>
-      <c r="D45" s="78" t="s">
-        <v>332</v>
-      </c>
-      <c r="E45" s="79"/>
-      <c r="F45" s="34" t="s">
-        <v>337</v>
-      </c>
-      <c r="G45" s="35"/>
-      <c r="H45" s="50" t="s">
+      <c r="B46" s="78" t="s">
+        <v>329</v>
+      </c>
+      <c r="C46" s="79"/>
+      <c r="D46" s="78" t="s">
+        <v>330</v>
+      </c>
+      <c r="E46" s="79"/>
+      <c r="F46" s="34" t="s">
+        <v>335</v>
+      </c>
+      <c r="G46" s="35"/>
+      <c r="H46" s="50" t="s">
         <v>275</v>
       </c>
-      <c r="I45" s="51"/>
-      <c r="J45" s="50" t="s">
+      <c r="I46" s="51"/>
+      <c r="J46" s="50" t="s">
         <v>275</v>
       </c>
-      <c r="K45" s="51"/>
-      <c r="N45" s="6" t="s">
+      <c r="K46" s="51"/>
+      <c r="N46" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="O45" s="105" t="s">
-        <v>323</v>
-      </c>
-      <c r="P45" s="106"/>
-      <c r="Q45" s="105" t="s">
-        <v>323</v>
-      </c>
-      <c r="R45" s="106"/>
-      <c r="S45" s="24" t="s">
+      <c r="O46" s="105" t="s">
+        <v>321</v>
+      </c>
+      <c r="P46" s="106"/>
+      <c r="Q46" s="105" t="s">
+        <v>321</v>
+      </c>
+      <c r="R46" s="106"/>
+      <c r="S46" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="T45" s="25"/>
-      <c r="U45" s="24" t="s">
+      <c r="T46" s="25"/>
+      <c r="U46" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="V45" s="25"/>
-      <c r="W45" s="46" t="s">
+      <c r="V46" s="25"/>
+      <c r="W46" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="X45" s="47"/>
-    </row>
-    <row r="46" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A46" s="6" t="s">
+      <c r="X46" s="47"/>
+    </row>
+    <row r="47" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A47" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B46" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="C46" s="21"/>
-      <c r="D46" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="E46" s="21"/>
-      <c r="F46" s="46" t="s">
+      <c r="B47" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="C47" s="21"/>
+      <c r="D47" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="E47" s="21"/>
+      <c r="F47" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="G46" s="47"/>
-      <c r="H46" s="34" t="s">
-        <v>337</v>
-      </c>
-      <c r="I46" s="35"/>
-      <c r="J46" s="46" t="s">
+      <c r="G47" s="47"/>
+      <c r="H47" s="34" t="s">
+        <v>335</v>
+      </c>
+      <c r="I47" s="35"/>
+      <c r="J47" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="K46" s="47"/>
-      <c r="L46" s="7"/>
-      <c r="M46" s="7"/>
-      <c r="N46" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="O46" s="44" t="s">
-        <v>91</v>
-      </c>
-      <c r="P46" s="45"/>
-      <c r="Q46" s="44" t="s">
-        <v>91</v>
-      </c>
-      <c r="R46" s="45"/>
-      <c r="S46" s="44" t="s">
-        <v>91</v>
-      </c>
-      <c r="T46" s="45"/>
-      <c r="U46" s="44" t="s">
-        <v>91</v>
-      </c>
-      <c r="V46" s="45"/>
-      <c r="W46" s="44" t="s">
-        <v>91</v>
-      </c>
-      <c r="X46" s="45"/>
-    </row>
-    <row r="47" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A47" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B47" s="34" t="s">
-        <v>350</v>
-      </c>
-      <c r="C47" s="35"/>
-      <c r="D47" s="34" t="s">
-        <v>351</v>
-      </c>
-      <c r="E47" s="35"/>
-      <c r="F47" s="34" t="s">
-        <v>351</v>
-      </c>
-      <c r="G47" s="35"/>
-      <c r="H47" s="34" t="s">
-        <v>351</v>
-      </c>
-      <c r="I47" s="35"/>
-      <c r="J47" s="34" t="s">
-        <v>351</v>
-      </c>
-      <c r="K47" s="35"/>
+      <c r="K47" s="47"/>
       <c r="L47" s="7"/>
       <c r="M47" s="7"/>
-      <c r="N47" s="1" t="s">
+      <c r="N47" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="O47" s="44" t="s">
+        <v>91</v>
+      </c>
+      <c r="P47" s="45"/>
+      <c r="Q47" s="44" t="s">
+        <v>91</v>
+      </c>
+      <c r="R47" s="45"/>
+      <c r="S47" s="44" t="s">
+        <v>91</v>
+      </c>
+      <c r="T47" s="45"/>
+      <c r="U47" s="44" t="s">
+        <v>91</v>
+      </c>
+      <c r="V47" s="45"/>
+      <c r="W47" s="44" t="s">
+        <v>91</v>
+      </c>
+      <c r="X47" s="45"/>
+    </row>
+    <row r="48" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A48" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="O47" s="105" t="s">
-        <v>354</v>
-      </c>
-      <c r="P47" s="106"/>
-      <c r="Q47" s="105" t="s">
-        <v>354</v>
-      </c>
-      <c r="R47" s="106"/>
-      <c r="S47" s="34" t="s">
-        <v>355</v>
-      </c>
-      <c r="T47" s="35"/>
-      <c r="U47" s="34" t="s">
-        <v>355</v>
-      </c>
-      <c r="V47" s="35"/>
-      <c r="W47" s="34" t="s">
-        <v>355</v>
-      </c>
-      <c r="X47" s="35"/>
-    </row>
-    <row r="48" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B48" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="C48" s="21"/>
+      <c r="B48" s="34" t="s">
+        <v>348</v>
+      </c>
+      <c r="C48" s="35"/>
       <c r="D48" s="34" t="s">
-        <v>103</v>
+        <v>349</v>
       </c>
       <c r="E48" s="35"/>
       <c r="F48" s="34" t="s">
-        <v>103</v>
+        <v>349</v>
       </c>
       <c r="G48" s="35"/>
       <c r="H48" s="34" t="s">
-        <v>103</v>
+        <v>349</v>
       </c>
       <c r="I48" s="35"/>
       <c r="J48" s="34" t="s">
-        <v>103</v>
+        <v>349</v>
       </c>
       <c r="K48" s="35"/>
       <c r="L48" s="7"/>
       <c r="M48" s="7"/>
       <c r="N48" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="O48" s="105" t="s">
+        <v>352</v>
+      </c>
+      <c r="P48" s="106"/>
+      <c r="Q48" s="105" t="s">
+        <v>352</v>
+      </c>
+      <c r="R48" s="106"/>
+      <c r="S48" s="34" t="s">
+        <v>353</v>
+      </c>
+      <c r="T48" s="35"/>
+      <c r="U48" s="34" t="s">
+        <v>353</v>
+      </c>
+      <c r="V48" s="35"/>
+      <c r="W48" s="34" t="s">
+        <v>353</v>
+      </c>
+      <c r="X48" s="35"/>
+    </row>
+    <row r="49" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="O48" s="44" t="s">
-        <v>91</v>
-      </c>
-      <c r="P48" s="45"/>
-      <c r="Q48" s="44" t="s">
-        <v>91</v>
-      </c>
-      <c r="R48" s="45"/>
-      <c r="S48" s="44" t="s">
-        <v>91</v>
-      </c>
-      <c r="T48" s="45"/>
-      <c r="U48" s="44" t="s">
-        <v>91</v>
-      </c>
-      <c r="V48" s="45"/>
-      <c r="W48" s="44" t="s">
-        <v>91</v>
-      </c>
-      <c r="X48" s="45"/>
-    </row>
-    <row r="49" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A49" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="B49" s="34" t="s">
-        <v>317</v>
-      </c>
-      <c r="C49" s="35"/>
+      <c r="B49" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="C49" s="21"/>
       <c r="D49" s="34" t="s">
-        <v>301</v>
+        <v>103</v>
       </c>
       <c r="E49" s="35"/>
       <c r="F49" s="34" t="s">
-        <v>301</v>
+        <v>103</v>
       </c>
       <c r="G49" s="35"/>
       <c r="H49" s="34" t="s">
-        <v>301</v>
+        <v>103</v>
       </c>
       <c r="I49" s="35"/>
       <c r="J49" s="34" t="s">
-        <v>301</v>
+        <v>103</v>
       </c>
       <c r="K49" s="35"/>
       <c r="L49" s="7"/>
       <c r="M49" s="7"/>
-      <c r="N49" s="12" t="s">
+      <c r="N49" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="O49" s="44" t="s">
+        <v>91</v>
+      </c>
+      <c r="P49" s="45"/>
+      <c r="Q49" s="44" t="s">
+        <v>91</v>
+      </c>
+      <c r="R49" s="45"/>
+      <c r="S49" s="44" t="s">
+        <v>91</v>
+      </c>
+      <c r="T49" s="45"/>
+      <c r="U49" s="44" t="s">
+        <v>91</v>
+      </c>
+      <c r="V49" s="45"/>
+      <c r="W49" s="44" t="s">
+        <v>91</v>
+      </c>
+      <c r="X49" s="45"/>
+    </row>
+    <row r="50" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A50" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="O49" s="46" t="s">
+      <c r="B50" s="34" t="s">
+        <v>316</v>
+      </c>
+      <c r="C50" s="35"/>
+      <c r="D50" s="34" t="s">
+        <v>300</v>
+      </c>
+      <c r="E50" s="35"/>
+      <c r="F50" s="34" t="s">
+        <v>300</v>
+      </c>
+      <c r="G50" s="35"/>
+      <c r="H50" s="34" t="s">
+        <v>300</v>
+      </c>
+      <c r="I50" s="35"/>
+      <c r="J50" s="34" t="s">
+        <v>300</v>
+      </c>
+      <c r="K50" s="35"/>
+      <c r="L50" s="7"/>
+      <c r="M50" s="7"/>
+      <c r="N50" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="O50" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="P49" s="47"/>
-      <c r="Q49" s="46" t="s">
+      <c r="P50" s="47"/>
+      <c r="Q50" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="R49" s="47"/>
-      <c r="S49" s="34" t="s">
-        <v>356</v>
-      </c>
-      <c r="T49" s="35"/>
-      <c r="U49" s="34" t="s">
-        <v>356</v>
-      </c>
-      <c r="V49" s="35"/>
-      <c r="W49" s="34" t="s">
-        <v>356</v>
-      </c>
-      <c r="X49" s="35"/>
-    </row>
-    <row r="50" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="1" t="s">
+      <c r="R50" s="47"/>
+      <c r="S50" s="34" t="s">
+        <v>354</v>
+      </c>
+      <c r="T50" s="35"/>
+      <c r="U50" s="34" t="s">
+        <v>354</v>
+      </c>
+      <c r="V50" s="35"/>
+      <c r="W50" s="34" t="s">
+        <v>354</v>
+      </c>
+      <c r="X50" s="35"/>
+    </row>
+    <row r="51" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B50" s="46" t="s">
+      <c r="B51" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="C50" s="47"/>
-      <c r="D50" s="50" t="s">
+      <c r="C51" s="47"/>
+      <c r="D51" s="50" t="s">
         <v>286</v>
       </c>
-      <c r="E50" s="51"/>
-      <c r="F50" s="46" t="s">
+      <c r="E51" s="51"/>
+      <c r="F51" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="G50" s="47"/>
-      <c r="H50" s="50" t="s">
+      <c r="G51" s="47"/>
+      <c r="H51" s="50" t="s">
         <v>286</v>
       </c>
-      <c r="I50" s="51"/>
-      <c r="J50" s="50" t="s">
+      <c r="I51" s="51"/>
+      <c r="J51" s="50" t="s">
         <v>286</v>
       </c>
-      <c r="K50" s="51"/>
-      <c r="N50" s="1" t="s">
+      <c r="K51" s="51"/>
+      <c r="N51" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="O50" s="76" t="s">
+      <c r="O51" s="76" t="s">
         <v>186</v>
-      </c>
-      <c r="P50" s="77"/>
-      <c r="Q50" s="76" t="s">
-        <v>186</v>
-      </c>
-      <c r="R50" s="77"/>
-      <c r="S50" s="76" t="s">
-        <v>186</v>
-      </c>
-      <c r="T50" s="77"/>
-      <c r="U50" s="76" t="s">
-        <v>186</v>
-      </c>
-      <c r="V50" s="77"/>
-      <c r="W50" s="76" t="s">
-        <v>186</v>
-      </c>
-      <c r="X50" s="77"/>
-    </row>
-    <row r="51" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A51" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="B51" s="34" t="s">
-        <v>348</v>
-      </c>
-      <c r="C51" s="35"/>
-      <c r="D51" s="34" t="s">
-        <v>349</v>
-      </c>
-      <c r="E51" s="35"/>
-      <c r="F51" s="34" t="s">
-        <v>349</v>
-      </c>
-      <c r="G51" s="35"/>
-      <c r="H51" s="34" t="s">
-        <v>349</v>
-      </c>
-      <c r="I51" s="35"/>
-      <c r="J51" s="34" t="s">
-        <v>349</v>
-      </c>
-      <c r="K51" s="35"/>
-      <c r="N51" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="O51" s="76" t="s">
-        <v>183</v>
       </c>
       <c r="P51" s="77"/>
       <c r="Q51" s="76" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="R51" s="77"/>
       <c r="S51" s="76" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="T51" s="77"/>
       <c r="U51" s="76" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="V51" s="77"/>
       <c r="W51" s="76" t="s">
+        <v>186</v>
+      </c>
+      <c r="X51" s="77"/>
+    </row>
+    <row r="52" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A52" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="B52" s="34" t="s">
+        <v>346</v>
+      </c>
+      <c r="C52" s="35"/>
+      <c r="D52" s="34" t="s">
+        <v>347</v>
+      </c>
+      <c r="E52" s="35"/>
+      <c r="F52" s="34" t="s">
+        <v>347</v>
+      </c>
+      <c r="G52" s="35"/>
+      <c r="H52" s="34" t="s">
+        <v>347</v>
+      </c>
+      <c r="I52" s="35"/>
+      <c r="J52" s="34" t="s">
+        <v>347</v>
+      </c>
+      <c r="K52" s="35"/>
+      <c r="N52" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="O52" s="76" t="s">
         <v>183</v>
       </c>
-      <c r="X51" s="77"/>
-    </row>
-    <row r="52" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A52" s="1" t="s">
+      <c r="P52" s="77"/>
+      <c r="Q52" s="76" t="s">
+        <v>183</v>
+      </c>
+      <c r="R52" s="77"/>
+      <c r="S52" s="76" t="s">
+        <v>183</v>
+      </c>
+      <c r="T52" s="77"/>
+      <c r="U52" s="76" t="s">
+        <v>183</v>
+      </c>
+      <c r="V52" s="77"/>
+      <c r="W52" s="76" t="s">
+        <v>183</v>
+      </c>
+      <c r="X52" s="77"/>
+    </row>
+    <row r="53" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A53" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B52" s="78" t="s">
-        <v>352</v>
-      </c>
-      <c r="C52" s="79"/>
-      <c r="D52" s="78" t="s">
-        <v>353</v>
-      </c>
-      <c r="E52" s="79"/>
-      <c r="F52" s="20" t="s">
+      <c r="B53" s="78" t="s">
+        <v>350</v>
+      </c>
+      <c r="C53" s="79"/>
+      <c r="D53" s="78" t="s">
+        <v>351</v>
+      </c>
+      <c r="E53" s="79"/>
+      <c r="F53" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="G52" s="21"/>
-      <c r="H52" s="46" t="s">
+      <c r="G53" s="21"/>
+      <c r="H53" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="I52" s="47"/>
-      <c r="J52" s="46" t="s">
+      <c r="I53" s="47"/>
+      <c r="J53" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="K52" s="47"/>
-      <c r="N52" s="1" t="s">
+      <c r="K53" s="47"/>
+      <c r="N53" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="O52" s="24" t="s">
+      <c r="O53" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="P52" s="25"/>
-      <c r="Q52" s="24" t="s">
+      <c r="P53" s="25"/>
+      <c r="Q53" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="R52" s="25"/>
-      <c r="S52" s="20" t="s">
+      <c r="R53" s="25"/>
+      <c r="S53" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="T52" s="21"/>
-      <c r="U52" s="24" t="s">
+      <c r="T53" s="21"/>
+      <c r="U53" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="V52" s="25"/>
-      <c r="W52" s="24" t="s">
+      <c r="V53" s="25"/>
+      <c r="W53" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="X52" s="25"/>
-    </row>
-    <row r="54" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A54" s="5">
-        <v>1</v>
-      </c>
-      <c r="B54" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="G54" s="5">
-        <v>5</v>
-      </c>
-      <c r="H54" s="5" t="s">
-        <v>80</v>
-      </c>
+      <c r="X53" s="25"/>
     </row>
     <row r="55" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A55" s="5">
+        <v>1</v>
+      </c>
+      <c r="B55" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="G55" s="5">
+        <v>5</v>
+      </c>
+      <c r="H55" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="56" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A56" s="5">
         <v>2</v>
       </c>
-      <c r="B55" s="5" t="s">
+      <c r="B56" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="G55" s="8">
+      <c r="G56" s="8">
         <v>6</v>
       </c>
-      <c r="H55" s="4" t="s">
+      <c r="H56" s="4" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="56" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A56" s="8">
+    <row r="57" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A57" s="8">
         <v>3</v>
       </c>
-      <c r="B56" s="5" t="s">
+      <c r="B57" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="C56" s="5"/>
-      <c r="G56" s="8">
-        <v>9</v>
-      </c>
-      <c r="H56" s="4" t="s">
+      <c r="C57" s="5"/>
+      <c r="G57" s="8">
+        <v>9</v>
+      </c>
+      <c r="H57" s="4" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="57" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A57" s="5">
+    <row r="58" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A58" s="5">
         <v>4</v>
       </c>
-      <c r="B57" s="4" t="s">
+      <c r="B58" s="4" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="58" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A58" s="5"/>
-      <c r="B58" s="5"/>
-      <c r="C58" s="5"/>
     </row>
     <row r="59" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A59" s="5"/>
@@ -26532,9 +26560,14 @@
       <c r="B60" s="5"/>
       <c r="C60" s="5"/>
     </row>
+    <row r="61" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A61" s="5"/>
+      <c r="B61" s="5"/>
+      <c r="C61" s="5"/>
+    </row>
   </sheetData>
-  <mergeCells count="450">
-    <mergeCell ref="U42:V42"/>
+  <mergeCells count="451">
+    <mergeCell ref="U43:V43"/>
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="D33:E33"/>
     <mergeCell ref="F33:G33"/>
@@ -26544,44 +26577,44 @@
     <mergeCell ref="Q33:R33"/>
     <mergeCell ref="S33:T33"/>
     <mergeCell ref="U33:V33"/>
-    <mergeCell ref="S42:T42"/>
-    <mergeCell ref="Q38:R38"/>
-    <mergeCell ref="S38:T38"/>
-    <mergeCell ref="U38:V38"/>
+    <mergeCell ref="S43:T43"/>
+    <mergeCell ref="Q39:R39"/>
+    <mergeCell ref="S39:T39"/>
+    <mergeCell ref="U39:V39"/>
+    <mergeCell ref="O41:P41"/>
+    <mergeCell ref="Q41:R41"/>
+    <mergeCell ref="S41:T41"/>
+    <mergeCell ref="U41:V41"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="H40:I40"/>
+    <mergeCell ref="J40:K40"/>
     <mergeCell ref="O40:P40"/>
     <mergeCell ref="Q40:R40"/>
-    <mergeCell ref="S40:T40"/>
-    <mergeCell ref="U40:V40"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="H39:I39"/>
-    <mergeCell ref="J39:K39"/>
-    <mergeCell ref="O39:P39"/>
-    <mergeCell ref="Q39:R39"/>
-    <mergeCell ref="B50:C50"/>
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="F50:G50"/>
-    <mergeCell ref="W51:X51"/>
     <mergeCell ref="B51:C51"/>
     <mergeCell ref="D51:E51"/>
     <mergeCell ref="F51:G51"/>
-    <mergeCell ref="F43:G43"/>
-    <mergeCell ref="J51:K51"/>
-    <mergeCell ref="O51:P51"/>
-    <mergeCell ref="Q51:R51"/>
-    <mergeCell ref="S51:T51"/>
-    <mergeCell ref="U51:V51"/>
-    <mergeCell ref="W47:X47"/>
-    <mergeCell ref="O48:P48"/>
-    <mergeCell ref="Q48:R48"/>
-    <mergeCell ref="S48:T48"/>
-    <mergeCell ref="U48:V48"/>
-    <mergeCell ref="W50:X50"/>
-    <mergeCell ref="O47:P47"/>
-    <mergeCell ref="Q47:R47"/>
+    <mergeCell ref="W52:X52"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="F52:G52"/>
+    <mergeCell ref="F44:G44"/>
+    <mergeCell ref="J52:K52"/>
+    <mergeCell ref="O52:P52"/>
+    <mergeCell ref="Q52:R52"/>
+    <mergeCell ref="S52:T52"/>
+    <mergeCell ref="U52:V52"/>
     <mergeCell ref="W48:X48"/>
     <mergeCell ref="O49:P49"/>
     <mergeCell ref="Q49:R49"/>
+    <mergeCell ref="S49:T49"/>
+    <mergeCell ref="U49:V49"/>
+    <mergeCell ref="W51:X51"/>
+    <mergeCell ref="O48:P48"/>
+    <mergeCell ref="Q48:R48"/>
+    <mergeCell ref="W49:X49"/>
+    <mergeCell ref="O50:P50"/>
+    <mergeCell ref="Q50:R50"/>
     <mergeCell ref="B32:C32"/>
     <mergeCell ref="D32:E32"/>
     <mergeCell ref="F32:G32"/>
@@ -26615,44 +26648,44 @@
     <mergeCell ref="Q15:R15"/>
     <mergeCell ref="S15:T15"/>
     <mergeCell ref="U15:V15"/>
-    <mergeCell ref="W49:X49"/>
-    <mergeCell ref="O43:P43"/>
-    <mergeCell ref="Q43:R43"/>
-    <mergeCell ref="U45:V45"/>
-    <mergeCell ref="S45:T45"/>
-    <mergeCell ref="W46:X46"/>
+    <mergeCell ref="W50:X50"/>
+    <mergeCell ref="O44:P44"/>
+    <mergeCell ref="Q44:R44"/>
+    <mergeCell ref="U46:V46"/>
+    <mergeCell ref="S46:T46"/>
+    <mergeCell ref="W47:X47"/>
+    <mergeCell ref="O47:P47"/>
+    <mergeCell ref="Q47:R47"/>
+    <mergeCell ref="S47:T47"/>
+    <mergeCell ref="U47:V47"/>
+    <mergeCell ref="W44:X44"/>
     <mergeCell ref="O46:P46"/>
     <mergeCell ref="Q46:R46"/>
-    <mergeCell ref="S46:T46"/>
-    <mergeCell ref="U46:V46"/>
-    <mergeCell ref="W43:X43"/>
+    <mergeCell ref="W45:X45"/>
+    <mergeCell ref="W46:X46"/>
+    <mergeCell ref="S44:T44"/>
+    <mergeCell ref="S45:T45"/>
+    <mergeCell ref="U45:V45"/>
     <mergeCell ref="O45:P45"/>
     <mergeCell ref="Q45:R45"/>
-    <mergeCell ref="W44:X44"/>
-    <mergeCell ref="W45:X45"/>
-    <mergeCell ref="S43:T43"/>
-    <mergeCell ref="S44:T44"/>
-    <mergeCell ref="U44:V44"/>
-    <mergeCell ref="O44:P44"/>
-    <mergeCell ref="Q44:R44"/>
-    <mergeCell ref="H50:I50"/>
-    <mergeCell ref="J50:K50"/>
-    <mergeCell ref="O50:P50"/>
-    <mergeCell ref="Q50:R50"/>
+    <mergeCell ref="H51:I51"/>
+    <mergeCell ref="J51:K51"/>
+    <mergeCell ref="O51:P51"/>
+    <mergeCell ref="Q51:R51"/>
+    <mergeCell ref="S51:T51"/>
+    <mergeCell ref="U51:V51"/>
+    <mergeCell ref="U48:V48"/>
+    <mergeCell ref="H48:I48"/>
+    <mergeCell ref="J48:K48"/>
+    <mergeCell ref="S48:T48"/>
     <mergeCell ref="S50:T50"/>
     <mergeCell ref="U50:V50"/>
-    <mergeCell ref="U47:V47"/>
-    <mergeCell ref="H47:I47"/>
-    <mergeCell ref="J47:K47"/>
-    <mergeCell ref="S47:T47"/>
-    <mergeCell ref="S49:T49"/>
-    <mergeCell ref="U49:V49"/>
-    <mergeCell ref="J48:K48"/>
-    <mergeCell ref="W40:X40"/>
-    <mergeCell ref="O41:P41"/>
-    <mergeCell ref="Q41:R41"/>
-    <mergeCell ref="S41:T41"/>
-    <mergeCell ref="U41:V41"/>
+    <mergeCell ref="J49:K49"/>
+    <mergeCell ref="W41:X41"/>
+    <mergeCell ref="O42:P42"/>
+    <mergeCell ref="Q42:R42"/>
+    <mergeCell ref="S42:T42"/>
+    <mergeCell ref="U42:V42"/>
     <mergeCell ref="O31:P31"/>
     <mergeCell ref="Q31:R31"/>
     <mergeCell ref="S31:T31"/>
@@ -26661,16 +26694,17 @@
     <mergeCell ref="W32:X32"/>
     <mergeCell ref="U32:V32"/>
     <mergeCell ref="W33:X33"/>
-    <mergeCell ref="W38:X38"/>
-    <mergeCell ref="W41:X41"/>
-    <mergeCell ref="S39:T39"/>
-    <mergeCell ref="U39:V39"/>
     <mergeCell ref="W39:X39"/>
+    <mergeCell ref="W42:X42"/>
+    <mergeCell ref="S40:T40"/>
+    <mergeCell ref="U40:V40"/>
+    <mergeCell ref="W40:X40"/>
     <mergeCell ref="W34:X34"/>
     <mergeCell ref="O34:P34"/>
     <mergeCell ref="Q34:R34"/>
     <mergeCell ref="S34:T34"/>
     <mergeCell ref="U34:V34"/>
+    <mergeCell ref="O35:P35"/>
     <mergeCell ref="O12:P12"/>
     <mergeCell ref="S12:T12"/>
     <mergeCell ref="U12:V12"/>
@@ -26821,11 +26855,11 @@
     <mergeCell ref="O3:P3"/>
     <mergeCell ref="Q3:R3"/>
     <mergeCell ref="F9:G9"/>
-    <mergeCell ref="Q42:R42"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="H42:I42"/>
-    <mergeCell ref="J42:K42"/>
-    <mergeCell ref="O42:P42"/>
+    <mergeCell ref="Q43:R43"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="J43:K43"/>
+    <mergeCell ref="O43:P43"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="F2:G2"/>
@@ -26845,18 +26879,18 @@
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="Q23:R23"/>
-    <mergeCell ref="W42:X42"/>
-    <mergeCell ref="O38:P38"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="F47:G47"/>
+    <mergeCell ref="W43:X43"/>
+    <mergeCell ref="O39:P39"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="F48:G48"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="D3:E3"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="H3:I3"/>
     <mergeCell ref="J3:K3"/>
-    <mergeCell ref="U43:V43"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="U44:V44"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="D45:E45"/>
     <mergeCell ref="Q12:R12"/>
     <mergeCell ref="S10:T10"/>
     <mergeCell ref="O10:P10"/>
@@ -26868,8 +26902,8 @@
     <mergeCell ref="F8:G8"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="D9:E9"/>
-    <mergeCell ref="J40:K40"/>
-    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="J41:K41"/>
+    <mergeCell ref="F42:G42"/>
     <mergeCell ref="B22:C22"/>
     <mergeCell ref="D22:E22"/>
     <mergeCell ref="F22:G22"/>
@@ -26894,25 +26928,25 @@
     <mergeCell ref="D24:E24"/>
     <mergeCell ref="H9:I9"/>
     <mergeCell ref="J9:K9"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="F44:G44"/>
-    <mergeCell ref="H44:I44"/>
-    <mergeCell ref="J44:K44"/>
-    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="F45:G45"/>
+    <mergeCell ref="H45:I45"/>
+    <mergeCell ref="J45:K45"/>
+    <mergeCell ref="D43:E43"/>
     <mergeCell ref="H27:I27"/>
     <mergeCell ref="D28:E28"/>
     <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J38:K38"/>
-    <mergeCell ref="H40:I40"/>
-    <mergeCell ref="H38:I38"/>
-    <mergeCell ref="F40:G40"/>
-    <mergeCell ref="H43:I43"/>
-    <mergeCell ref="J43:K43"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="J39:K39"/>
+    <mergeCell ref="H41:I41"/>
+    <mergeCell ref="H39:I39"/>
+    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="H44:I44"/>
+    <mergeCell ref="J44:K44"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="D39:E39"/>
     <mergeCell ref="B42:C42"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="B43:C43"/>
     <mergeCell ref="H29:I29"/>
     <mergeCell ref="H26:I26"/>
     <mergeCell ref="H28:I28"/>
@@ -26931,59 +26965,59 @@
     <mergeCell ref="J26:K26"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="D20:E20"/>
-    <mergeCell ref="H51:I51"/>
-    <mergeCell ref="H41:I41"/>
-    <mergeCell ref="J41:K41"/>
-    <mergeCell ref="F42:G42"/>
+    <mergeCell ref="H52:I52"/>
+    <mergeCell ref="H42:I42"/>
+    <mergeCell ref="J42:K42"/>
+    <mergeCell ref="F43:G43"/>
     <mergeCell ref="H34:I34"/>
     <mergeCell ref="J34:K34"/>
     <mergeCell ref="H21:I21"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="D27:E27"/>
     <mergeCell ref="F27:G27"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="F45:G45"/>
-    <mergeCell ref="H45:I45"/>
-    <mergeCell ref="J45:K45"/>
-    <mergeCell ref="B46:C46"/>
     <mergeCell ref="D46:E46"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="H46:I46"/>
+    <mergeCell ref="J46:K46"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="F40:G40"/>
     <mergeCell ref="F39:G39"/>
-    <mergeCell ref="F38:G38"/>
-    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="B44:C44"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="D16:E16"/>
     <mergeCell ref="F16:G16"/>
     <mergeCell ref="H16:I16"/>
     <mergeCell ref="J16:K16"/>
     <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B50:C50"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="F50:G50"/>
+    <mergeCell ref="H50:I50"/>
+    <mergeCell ref="J50:K50"/>
+    <mergeCell ref="F47:G47"/>
+    <mergeCell ref="H47:I47"/>
+    <mergeCell ref="J47:K47"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B48:C48"/>
     <mergeCell ref="B49:C49"/>
     <mergeCell ref="D49:E49"/>
     <mergeCell ref="F49:G49"/>
     <mergeCell ref="H49:I49"/>
-    <mergeCell ref="J49:K49"/>
-    <mergeCell ref="F46:G46"/>
-    <mergeCell ref="H46:I46"/>
-    <mergeCell ref="J46:K46"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="F48:G48"/>
-    <mergeCell ref="H48:I48"/>
-    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="D41:E41"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="D34:E34"/>
     <mergeCell ref="F34:G34"/>
-    <mergeCell ref="W52:X52"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="F52:G52"/>
-    <mergeCell ref="H52:I52"/>
-    <mergeCell ref="J52:K52"/>
-    <mergeCell ref="O52:P52"/>
-    <mergeCell ref="Q52:R52"/>
-    <mergeCell ref="S52:T52"/>
-    <mergeCell ref="U52:V52"/>
+    <mergeCell ref="W53:X53"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="F53:G53"/>
+    <mergeCell ref="H53:I53"/>
+    <mergeCell ref="J53:K53"/>
+    <mergeCell ref="O53:P53"/>
+    <mergeCell ref="Q53:R53"/>
+    <mergeCell ref="S53:T53"/>
+    <mergeCell ref="U53:V53"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -27033,7 +27067,7 @@
     <row r="1" spans="2:25" ht="6.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="2" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>1</v>
@@ -27066,7 +27100,7 @@
         <v>46360</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>1</v>
@@ -27306,11 +27340,11 @@
         <v>26</v>
       </c>
       <c r="C8" s="34" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="D8" s="35"/>
       <c r="E8" s="34" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="F8" s="35"/>
       <c r="G8" s="88"/>
@@ -27340,11 +27374,11 @@
         <v>28</v>
       </c>
       <c r="C9" s="34" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="D9" s="35"/>
       <c r="E9" s="34" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="F9" s="35"/>
       <c r="G9" s="74"/>
@@ -27481,8 +27515,10 @@
         <v>72</v>
       </c>
       <c r="J13" s="43"/>
-      <c r="K13" s="20"/>
-      <c r="L13" s="21"/>
+      <c r="K13" s="34" t="s">
+        <v>340</v>
+      </c>
+      <c r="L13" s="35"/>
       <c r="O13" s="1" t="s">
         <v>40</v>
       </c>
@@ -27540,36 +27576,44 @@
         <v>48</v>
       </c>
       <c r="C15" s="34" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="D15" s="35"/>
       <c r="E15" s="34" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="F15" s="35"/>
       <c r="G15" s="34" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="H15" s="35"/>
       <c r="I15" s="34" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="J15" s="35"/>
-      <c r="K15" s="34" t="s">
-        <v>342</v>
-      </c>
-      <c r="L15" s="35"/>
+      <c r="K15" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="L15" s="41"/>
       <c r="O15" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="P15" s="20"/>
-      <c r="Q15" s="21"/>
-      <c r="R15" s="20"/>
-      <c r="S15" s="21"/>
-      <c r="T15" s="20"/>
-      <c r="U15" s="21"/>
-      <c r="V15" s="20"/>
-      <c r="W15" s="21"/>
+      <c r="P15" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q15" s="41"/>
+      <c r="R15" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="S15" s="41"/>
+      <c r="T15" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="U15" s="41"/>
+      <c r="V15" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="W15" s="41"/>
       <c r="X15" s="66"/>
       <c r="Y15" s="67"/>
     </row>
@@ -27666,7 +27710,7 @@
     </row>
     <row r="20" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B20" s="1" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>1</v>
@@ -27699,7 +27743,7 @@
         <v>46367</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="P20" s="2" t="s">
         <v>1</v>
@@ -28264,7 +28308,7 @@
     </row>
     <row r="38" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B38" s="1" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>1</v>
@@ -28633,7 +28677,7 @@
       <c r="C50" s="74"/>
       <c r="D50" s="75"/>
       <c r="E50" s="44" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="F50" s="45"/>
       <c r="G50" s="74"/>

</xml_diff>